<commit_message>
Fix Excel repair prompt in slicer triage tool; add clear-all macro module
The source draft's PresetResponses table declared column name 'Draft
email body' while its header cell read 'Draft email body - edit this
yellow column'. Excel treats that mismatch as corruption, repairs the
workbook on open, and the repair strips formulas (which is why the
travel slicer produced no draft text). The header cell now matches the
column name exactly. Also strips stale cached formula results, adds an
on-sheet tip for clearing slicers, and ships an optional
ClearAllSlicers.bas VBA module since Excel has no macro-free clear-all.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SAZNBMXD3sMU2sN7hJCcLM
</commit_message>
<xml_diff>
--- a/Principal wellbeing email triage tool.xlsx
+++ b/Principal wellbeing email triage tool.xlsx
@@ -252,7 +252,7 @@
     <t xml:space="preserve">Pick a greeting and add a name, e.g. 'Good morning Damien,'</t>
   </si>
   <si>
-    <t xml:space="preserve">Select Yes, No or Maybe in the question slicers below - you do not need to answer every question; unanswered ones are simply left out of the draft. For recurring queries, pick a common response override instead. Then add a greeting, name and topic under 'Draft email reply' and copy the finished draft into Outlook.</t>
+    <t xml:space="preserve">Select Yes, No or Maybe in the question slicers below - you do not need to answer every question; unanswered ones are simply left out of the draft. For recurring queries, pick a common response override instead. Then add a greeting, name and topic under 'Draft email reply' and copy the finished draft into Outlook. To clear a slicer, click the funnel-with-x button in its top right corner.</t>
   </si>
   <si>
     <t xml:space="preserve">Edit the modular wording on the Response library tab and the recurring full responses on the Preset responses tab. The draft remains a starting point: add case-specific detail and confirm the final advice against current Ikon guidance before sending.</t>
@@ -2848,7 +2848,6 @@
       </c>
       <c r="B2">
         <f>SUBTOTAL(103,A2)</f>
-        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2857,7 +2856,6 @@
       </c>
       <c r="B3">
         <f>SUBTOTAL(103,A3)</f>
-        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2866,7 +2864,6 @@
       </c>
       <c r="B4">
         <f>SUBTOTAL(103,A4)</f>
-        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2883,7 +2880,6 @@
       </c>
       <c r="B7">
         <f>SUBTOTAL(103,A7)</f>
-        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2892,7 +2888,6 @@
       </c>
       <c r="B8">
         <f>SUBTOTAL(103,A8)</f>
-        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2901,7 +2896,6 @@
       </c>
       <c r="B9">
         <f>SUBTOTAL(103,A9)</f>
-        <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2918,7 +2912,6 @@
       </c>
       <c r="B12">
         <f>SUBTOTAL(103,A12)</f>
-        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2927,7 +2920,6 @@
       </c>
       <c r="B13">
         <f>SUBTOTAL(103,A13)</f>
-        <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2936,7 +2928,6 @@
       </c>
       <c r="B14">
         <f>SUBTOTAL(103,A14)</f>
-        <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2953,7 +2944,6 @@
       </c>
       <c r="B17">
         <f>SUBTOTAL(103,A17)</f>
-        <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2962,7 +2952,6 @@
       </c>
       <c r="B18">
         <f>SUBTOTAL(103,A18)</f>
-        <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2971,7 +2960,6 @@
       </c>
       <c r="B19">
         <f>SUBTOTAL(103,A19)</f>
-        <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2988,7 +2976,6 @@
       </c>
       <c r="B22">
         <f>SUBTOTAL(103,A22)</f>
-        <v>1</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2997,7 +2984,6 @@
       </c>
       <c r="B23">
         <f>SUBTOTAL(103,A23)</f>
-        <v>1</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3006,7 +2992,6 @@
       </c>
       <c r="B24">
         <f>SUBTOTAL(103,A24)</f>
-        <v>1</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3023,7 +3008,6 @@
       </c>
       <c r="B27">
         <f>SUBTOTAL(103,A27)</f>
-        <v>1</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3032,7 +3016,6 @@
       </c>
       <c r="B28">
         <f>SUBTOTAL(103,A28)</f>
-        <v>1</v>
       </c>
     </row>
     <row r="29" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3041,7 +3024,6 @@
       </c>
       <c r="B29">
         <f>SUBTOTAL(103,A29)</f>
-        <v>1</v>
       </c>
     </row>
     <row r="31" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3058,7 +3040,6 @@
       </c>
       <c r="B32">
         <f>SUBTOTAL(103,A32)</f>
-        <v>1</v>
       </c>
     </row>
     <row r="33" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3067,7 +3048,6 @@
       </c>
       <c r="B33">
         <f>SUBTOTAL(103,A33)</f>
-        <v>1</v>
       </c>
     </row>
     <row r="34" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3076,7 +3056,6 @@
       </c>
       <c r="B34">
         <f>SUBTOTAL(103,A34)</f>
-        <v>1</v>
       </c>
     </row>
     <row r="36" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3093,7 +3072,6 @@
       </c>
       <c r="B37">
         <f>SUBTOTAL(103,A37)</f>
-        <v>1</v>
       </c>
     </row>
     <row r="38" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3102,7 +3080,6 @@
       </c>
       <c r="B38">
         <f>SUBTOTAL(103,A38)</f>
-        <v>1</v>
       </c>
     </row>
     <row r="39" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3164,63 +3141,48 @@
     <row r="40" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="J40" t="str">
         <f>IF(SUM($B$2:$B$4)=1,INDEX($A$2:$A$4,MATCH(1,$B$2:$B$4,0)),"")</f>
-        <v/>
       </c>
       <c r="K40" t="str">
         <f>IF(SUM($B$7:$B$9)=1,INDEX($A$7:$A$9,MATCH(1,$B$7:$B$9,0)),"")</f>
-        <v/>
       </c>
       <c r="L40" t="str">
         <f>IF(SUM($B$12:$B$14)=1,INDEX($A$12:$A$14,MATCH(1,$B$12:$B$14,0)),"")</f>
-        <v/>
       </c>
       <c r="M40" t="str">
         <f>IF(SUM($B$17:$B$19)=1,INDEX($A$17:$A$19,MATCH(1,$B$17:$B$19,0)),"")</f>
-        <v/>
       </c>
       <c r="N40" t="str">
         <f>IF(SUM($B$22:$B$24)=1,INDEX($A$22:$A$24,MATCH(1,$B$22:$B$24,0)),"")</f>
-        <v/>
       </c>
       <c r="O40" t="str">
         <f>IF(SUM($B$27:$B$29)=1,INDEX($A$27:$A$29,MATCH(1,$B$27:$B$29,0)),"")</f>
-        <v/>
       </c>
       <c r="P40" t="str">
         <f>IF(SUM($B$32:$B$34)=1,INDEX($A$32:$A$34,MATCH(1,$B$32:$B$34,0)),"")</f>
-        <v/>
       </c>
       <c r="Q40" t="str">
         <f>IF(SUM($B$37:$B$38)=1,INDEX($A$37:$A$38,MATCH(1,$B$37:$B$38,0)),"")</f>
-        <v/>
       </c>
       <c r="R40" t="str">
         <f>IF($J$40="","",IFERROR(INDEX('Response library'!$D$2:$D$24,MATCH("Q1|"&amp;$J$40,'Response library'!$E$2:$E$24,0)),""))</f>
-        <v/>
       </c>
       <c r="S40" t="str">
         <f>IF($K$40="","",IFERROR(INDEX('Response library'!$D$2:$D$24,MATCH("Q2|"&amp;$K$40,'Response library'!$E$2:$E$24,0)),""))</f>
-        <v/>
       </c>
       <c r="T40" t="str">
         <f>IF($L$40="","",IFERROR(INDEX('Response library'!$D$2:$D$24,MATCH("Q3|"&amp;$L$40,'Response library'!$E$2:$E$24,0)),""))</f>
-        <v/>
       </c>
       <c r="U40" t="str">
         <f>IF($M$40="","",IFERROR(INDEX('Response library'!$D$2:$D$24,MATCH("Q4|"&amp;$M$40,'Response library'!$E$2:$E$24,0)),""))</f>
-        <v/>
       </c>
       <c r="V40" t="str">
         <f>IF($N$40="","",IFERROR(INDEX('Response library'!$D$2:$D$24,MATCH("Q5|"&amp;$N$40,'Response library'!$E$2:$E$24,0)),""))</f>
-        <v/>
       </c>
       <c r="W40" t="str">
         <f>IF($O$40="","",IFERROR(INDEX('Response library'!$D$2:$D$24,MATCH("Q6|"&amp;$O$40,'Response library'!$E$2:$E$24,0)),""))</f>
-        <v/>
       </c>
       <c r="X40" t="str">
         <f>IF($P$40="","",IFERROR(INDEX('Response library'!$D$2:$D$24,MATCH("Panel|"&amp;$P$40,'Response library'!$E$2:$E$24,0)),""))</f>
-        <v/>
       </c>
       <c r="Y40" t="str">
         <f>IF($Q$40="","",IFERROR(T(INDEX('Response library'!$D$2:$D$24,MATCH("Travel|"&amp;$Q$40,'Response library'!$E$2:$E$24,0))),""))</f>
@@ -3943,8 +3905,10 @@
       <c r="A5" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>131</v>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Draft email body</t>
+        </is>
       </c>
       <c r="C5" s="4" t="s">
         <v>64</v>

</xml_diff>

<commit_message>
Make Travel slicer structurally identical to the working question slicers
Travel was the only slicer table with two options instead of three - the
sole structural difference from the seven slicers confirmed working in
Excel. Adds a Maybe option to the Travel table and a matching
Travel|Maybe paragraph to the Response library, and shows an explanatory
message instead of an empty email body when the only selected answer
(Travel: No) intentionally contributes no wording.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SAZNBMXD3sMU2sN7hJCcLM
</commit_message>
<xml_diff>
--- a/Principal wellbeing email triage tool.xlsx
+++ b/Principal wellbeing email triage tool.xlsx
@@ -105,7 +105,7 @@
     <t>Does this align with the panel of wellbeing service providers?</t>
   </si>
   <si>
-    <t>Does this involve travel or accommodation?</t>
+    <t xml:space="preserve">Does this involve travel or accommodation?</t>
   </si>
   <si>
     <t xml:space="preserve">Tip: to clear a slicer, select the small red 'X' funnel button in its top right corner.</t>
@@ -1784,8 +1784,8 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{00000000-000C-0000-FFFF-FFFF07000000}" name="TravelSlicerSource" displayName="TravelSlicerSource" ref="A36:B38" totalsRowShown="0">
-  <autoFilter ref="A36:B38" xr:uid="{00000000-0009-0000-0100-000008000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{00000000-000C-0000-FFFF-FFFF07000000}" name="TravelSlicerSource" displayName="TravelSlicerSource" ref="A36:B39" totalsRowShown="0">
+  <autoFilter ref="A36:B39" xr:uid="{00000000-0009-0000-0100-000008000000}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0700-000001000000}" name="Travel"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0700-000002000000}" name="Visible row"/>
@@ -2164,7 +2164,7 @@
     </row>
     <row r="35" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B35" s="15" t="str">
-        <f>TRIM(IF($D$33="","Hi",$D$33)&amp;" "&amp;TRIM($E$33))&amp;","&amp;CHAR(10)&amp;CHAR(10)&amp;IF(TRIM($D$34)="","Thank you for reaching out regarding the principal wellbeing targeted funding.","Thank you for reaching out regarding "&amp;TRIM($D$34)&amp;".")&amp;CHAR(10)&amp;CHAR(10)&amp;IF('Preset responses'!$F$2&lt;&gt;"",'Preset responses'!$F$2,IF(COUNTIF('Pivot source data'!$J$40:$Q$40,"?*")=0,"[Select an answer in one or more question slicers above, or pick a common response override, to build the body of the email.]",'Pivot source data'!$AA$40))&amp;CHAR(10)&amp;CHAR(10)&amp;"If you have any further questions, please reach out again. You can contact Principal wellbeing expenditure support by phone on 9264 4201 or by email at whsw.staffwellbeing@education.wa.edu.au."&amp;CHAR(10)&amp;CHAR(10)&amp;"Kind regards,"</f>
+        <f>TRIM(IF($D$33="","Hi",$D$33)&amp;" "&amp;TRIM($E$33))&amp;","&amp;CHAR(10)&amp;CHAR(10)&amp;IF(TRIM($D$34)="","Thank you for reaching out regarding the principal wellbeing targeted funding.","Thank you for reaching out regarding "&amp;TRIM($D$34)&amp;".")&amp;CHAR(10)&amp;CHAR(10)&amp;IF('Preset responses'!$F$2&lt;&gt;"",'Preset responses'!$F$2,IF(COUNTIF('Pivot source data'!$J$40:$Q$40,"?*")=0,"[Select an answer in one or more question slicers above, or pick a common response override, to build the body of the email.]",IF('Pivot source data'!$AA$40="","[The answers selected so far do not add any wording to the email - answer more of the question slicers above.]",'Pivot source data'!$AA$40)))&amp;CHAR(10)&amp;CHAR(10)&amp;"If you have any further questions, please reach out again. You can contact Principal wellbeing expenditure support by phone on 9264 4201 or by email at whsw.staffwellbeing@education.wa.edu.au."&amp;CHAR(10)&amp;CHAR(10)&amp;"Kind regards,"</f>
       </c>
       <c r="C35" s="15"/>
       <c r="D35" s="15"/>
@@ -3083,6 +3083,12 @@
       </c>
     </row>
     <row r="39" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>67</v>
+      </c>
+      <c r="B39">
+        <f>SUBTOTAL(103,A39)</f>
+      </c>
       <c r="J39" t="s">
         <v>75</v>
       </c>
@@ -3161,7 +3167,7 @@
         <f>IF(SUM($B$32:$B$34)=1,INDEX($A$32:$A$34,MATCH(1,$B$32:$B$34,0)),"")</f>
       </c>
       <c r="Q40" t="str">
-        <f>IF(SUM($B$37:$B$38)=1,INDEX($A$37:$A$38,MATCH(1,$B$37:$B$38,0)),"")</f>
+        <f>IF(SUM($B$37:$B$39)=1,INDEX($A$37:$A$39,MATCH(1,$B$37:$B$39,0)),"")</f>
       </c>
       <c r="R40" t="str">
         <f>IF($J$40="","",IFERROR(INDEX('Response library'!$D$2:$D$24,MATCH("Q1|"&amp;$J$40,'Response library'!$E$2:$E$24,0)),""))</f>
@@ -3185,7 +3191,7 @@
         <f>IF($P$40="","",IFERROR(INDEX('Response library'!$D$2:$D$24,MATCH("Panel|"&amp;$P$40,'Response library'!$E$2:$E$24,0)),""))</f>
       </c>
       <c r="Y40" t="str">
-        <f>IF($Q$40="","",IFERROR(T(INDEX('Response library'!$D$2:$D$24,MATCH("Travel|"&amp;$Q$40,'Response library'!$E$2:$E$24,0))),""))</f>
+        <f>IF($Q$40="","",IFERROR(T(INDEX('Response library'!$D$2:$D$25,MATCH("Travel|"&amp;$Q$40,'Response library'!$E$2:$E$25,0))),""))</f>
       </c>
       <c r="Z40" t="str">
         <f>IF(COUNTIF($J$40:$O$40,"?*")=0,"",IF(COUNTIF($J$40:$O$40,"No")&gt;0,"To answer briefly: based on the decision-making framework, this expenditure does not appear to be appropriate. Please see the detail below.",IF(COUNTIF($J$40:$O$40,"Yes")=6,"To answer briefly: based on the decision-making framework, this expenditure is likely to be appropriate. Please see the detail below.","To answer briefly: we need a little more information before this expenditure can be confirmed as appropriate. Please see the detail below.")))</f>
@@ -3406,7 +3412,7 @@
   <sheetPr>
     <tabColor rgb="FFE5803A"/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -3847,8 +3853,27 @@
         <v>Travel|No</v>
       </c>
     </row>
+    <row r="25" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="D25" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">It is not yet clear whether travel or accommodation will be involved. If it is, it may be funded where it supports the eligible wellbeing activity, in line with the Official Travel Policy - please check the approval requirements with us before booking.</t>
+        </is>
+      </c>
+      <c r="E25" s="5">
+        <f>A25&amp;"|"&amp;C25</f>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E24" xr:uid="{00000000-0009-0000-0000-000005000000}"/>
+  <autoFilter ref="A1:E25" xr:uid="{00000000-0009-0000-0000-000005000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
   <headerFooter>

</xml_diff>